<commit_message>
fix(ui): correções de dashboard solicitadas
</commit_message>
<xml_diff>
--- a/Planejamento Previsto.xlsx
+++ b/Planejamento Previsto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Viana e Moura\Downloads\Planejamento Emissário - LD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8220EF3-7CC8-483E-AF06-A6444AE33F2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7169FE3A-BEAA-4ECC-AC5E-4DA9379B3AE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EEA59E8E-9647-43AC-97C3-E8656E227CAD}"/>
   </bookViews>
@@ -197,7 +197,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -283,11 +283,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -367,6 +378,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -986,7 +998,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="26">
-        <f>SUM(I4:U4)</f>
+        <f>SUM(I4:V4)</f>
         <v>800</v>
       </c>
       <c r="D4" s="21">
@@ -1025,7 +1037,7 @@
         <v>0</v>
       </c>
       <c r="Q4" s="2">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="R4" s="2">
         <v>100</v>
@@ -1037,9 +1049,11 @@
         <v>100</v>
       </c>
       <c r="U4" s="2">
+        <v>100</v>
+      </c>
+      <c r="V4" s="2">
         <v>66</v>
       </c>
-      <c r="V4" s="2"/>
       <c r="W4" s="13"/>
       <c r="X4" s="13"/>
       <c r="Y4" s="13"/>
@@ -1340,7 +1354,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="26">
-        <f>SUM(L8:Z8)</f>
+        <f>SUM(L8:Y8)</f>
         <v>422</v>
       </c>
       <c r="D8" s="21">
@@ -1375,7 +1389,7 @@
         <v>20</v>
       </c>
       <c r="Q8" s="2">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="R8" s="2">
         <v>30</v>
@@ -1389,7 +1403,9 @@
       <c r="U8" s="2">
         <v>30</v>
       </c>
-      <c r="V8" s="2"/>
+      <c r="V8" s="2">
+        <v>30</v>
+      </c>
       <c r="W8" s="2">
         <v>30</v>
       </c>
@@ -1397,10 +1413,7 @@
         <v>30</v>
       </c>
       <c r="Y8" s="2">
-        <v>30</v>
-      </c>
-      <c r="Z8" s="2">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="AA8" s="13"/>
       <c r="AB8" s="13"/>
@@ -1526,7 +1539,7 @@
       </c>
       <c r="C10" s="26">
         <f>SUM(M10:Z10)</f>
-        <v>63.29999999999999</v>
+        <v>63.3</v>
       </c>
       <c r="D10" s="21">
         <v>46084</v>
@@ -1558,7 +1571,7 @@
         <v>5</v>
       </c>
       <c r="Q10" s="3">
-        <v>4.8</v>
+        <v>1</v>
       </c>
       <c r="R10" s="3">
         <v>4.8</v>
@@ -1572,18 +1585,20 @@
       <c r="U10" s="3">
         <v>4.8</v>
       </c>
-      <c r="V10" s="3"/>
+      <c r="V10" s="3">
+        <v>4.8</v>
+      </c>
       <c r="W10" s="3">
         <v>4.8</v>
       </c>
       <c r="X10" s="3">
-        <v>4.8</v>
+        <v>4.57</v>
       </c>
       <c r="Y10" s="3">
-        <v>4.8</v>
-      </c>
-      <c r="Z10" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.57</v>
+      </c>
+      <c r="Z10" s="31">
+        <v>4.5599999999999996</v>
       </c>
       <c r="AA10" s="13"/>
       <c r="AB10" s="13"/>
@@ -1709,7 +1724,7 @@
       </c>
       <c r="C12" s="26">
         <f>SUM(N12:AA12)</f>
-        <v>63.199999999999989</v>
+        <v>63.29999999999999</v>
       </c>
       <c r="D12" s="21">
         <v>46085</v>
@@ -1739,7 +1754,7 @@
         <v>5</v>
       </c>
       <c r="Q12" s="3">
-        <v>4.8</v>
+        <v>1</v>
       </c>
       <c r="R12" s="3">
         <v>4.8</v>
@@ -1753,7 +1768,9 @@
       <c r="U12" s="3">
         <v>4.8</v>
       </c>
-      <c r="V12" s="3"/>
+      <c r="V12" s="3">
+        <v>4.8</v>
+      </c>
       <c r="W12" s="3">
         <v>4.8</v>
       </c>
@@ -1764,12 +1781,12 @@
         <v>4.8</v>
       </c>
       <c r="Z12" s="3">
-        <v>4.8</v>
+        <v>4.57</v>
       </c>
       <c r="AA12" s="3">
-        <v>5</v>
-      </c>
-      <c r="AB12" s="3"/>
+        <v>4.33</v>
+      </c>
+      <c r="AB12" s="13"/>
       <c r="AC12" s="13"/>
       <c r="AD12" s="13"/>
       <c r="AE12" s="13"/>
@@ -1891,7 +1908,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="26">
-        <f>SUM(L14:AA14)</f>
+        <f>SUM(L14:AB14)</f>
         <v>399.99999999999994</v>
       </c>
       <c r="D14" s="21">
@@ -1926,37 +1943,41 @@
         <v>6</v>
       </c>
       <c r="Q14" s="3">
-        <v>30.7</v>
+        <v>6</v>
       </c>
       <c r="R14" s="3">
-        <v>30.7</v>
+        <v>28.2</v>
       </c>
       <c r="S14" s="3">
-        <v>30.7</v>
+        <v>28.2</v>
       </c>
       <c r="T14" s="3">
-        <v>30.7</v>
+        <v>28.2</v>
       </c>
       <c r="U14" s="3">
-        <v>30.7</v>
-      </c>
-      <c r="V14" s="3"/>
+        <v>28.2</v>
+      </c>
+      <c r="V14" s="3">
+        <v>28.2</v>
+      </c>
       <c r="W14" s="3">
-        <v>30.7</v>
+        <v>28.2</v>
       </c>
       <c r="X14" s="3">
-        <v>30.7</v>
+        <v>28.2</v>
       </c>
       <c r="Y14" s="3">
-        <v>30.7</v>
+        <v>28.2</v>
       </c>
       <c r="Z14" s="3">
-        <v>30.7</v>
+        <v>28.2</v>
       </c>
       <c r="AA14" s="3">
-        <v>39.700000000000003</v>
-      </c>
-      <c r="AB14" s="3"/>
+        <v>28.2</v>
+      </c>
+      <c r="AB14" s="3">
+        <v>28</v>
+      </c>
       <c r="AC14" s="13"/>
       <c r="AD14" s="13"/>
       <c r="AE14" s="13"/>
@@ -2078,8 +2099,8 @@
         <v>1</v>
       </c>
       <c r="C16" s="26">
-        <f>SUM(L16:AA16)</f>
-        <v>400</v>
+        <f>SUM(L16:AB16)</f>
+        <v>399.99999999999994</v>
       </c>
       <c r="D16" s="21">
         <v>46085</v>
@@ -2113,37 +2134,41 @@
         <v>6</v>
       </c>
       <c r="Q16" s="3">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="R16" s="3">
-        <v>30</v>
+        <v>28.2</v>
       </c>
       <c r="S16" s="3">
-        <v>30</v>
+        <v>28.2</v>
       </c>
       <c r="T16" s="3">
-        <v>30</v>
+        <v>28.2</v>
       </c>
       <c r="U16" s="3">
-        <v>30</v>
-      </c>
-      <c r="V16" s="3"/>
+        <v>28.2</v>
+      </c>
+      <c r="V16" s="3">
+        <v>28.2</v>
+      </c>
       <c r="W16" s="3">
-        <v>30</v>
+        <v>28.2</v>
       </c>
       <c r="X16" s="3">
-        <v>30</v>
+        <v>28.2</v>
       </c>
       <c r="Y16" s="3">
-        <v>30</v>
+        <v>28.2</v>
       </c>
       <c r="Z16" s="3">
-        <v>36</v>
+        <v>28.2</v>
       </c>
       <c r="AA16" s="3">
-        <v>40</v>
-      </c>
-      <c r="AB16" s="3"/>
+        <v>28.2</v>
+      </c>
+      <c r="AB16" s="3">
+        <v>28</v>
+      </c>
       <c r="AC16" s="13"/>
       <c r="AD16" s="13"/>
       <c r="AE16" s="13"/>
@@ -2265,8 +2290,8 @@
         <v>1</v>
       </c>
       <c r="C18" s="26">
-        <f>SUM(P18:Y18)</f>
-        <v>4</v>
+        <f>SUM(P18:AB18)</f>
+        <v>5</v>
       </c>
       <c r="D18" s="21">
         <v>46090</v>
@@ -2307,10 +2332,10 @@
       </c>
       <c r="Y18" s="3"/>
       <c r="Z18" s="3"/>
-      <c r="AA18" s="3">
+      <c r="AA18" s="3"/>
+      <c r="AB18" s="3">
         <v>1</v>
       </c>
-      <c r="AB18" s="3"/>
       <c r="AC18" s="13"/>
       <c r="AD18" s="13"/>
       <c r="AE18" s="13"/>
@@ -2467,39 +2492,43 @@
         <v>6</v>
       </c>
       <c r="Q20" s="3">
-        <v>26.5</v>
+        <v>0</v>
       </c>
       <c r="R20" s="3">
-        <v>26.5</v>
+        <v>25.25</v>
       </c>
       <c r="S20" s="3">
-        <v>26.5</v>
+        <v>25.25</v>
       </c>
       <c r="T20" s="3">
-        <v>26.5</v>
+        <v>25.25</v>
       </c>
       <c r="U20" s="3">
-        <v>26.5</v>
-      </c>
-      <c r="V20" s="3"/>
+        <v>25.25</v>
+      </c>
+      <c r="V20" s="3">
+        <v>25.25</v>
+      </c>
       <c r="W20" s="3">
-        <v>26.5</v>
+        <v>25.25</v>
       </c>
       <c r="X20" s="3">
-        <v>26.5</v>
+        <v>25.25</v>
       </c>
       <c r="Y20" s="3">
-        <v>26.5</v>
+        <v>25.25</v>
       </c>
       <c r="Z20" s="3">
-        <v>26.5</v>
+        <v>25.25</v>
       </c>
       <c r="AA20" s="3">
-        <v>32.25</v>
-      </c>
-      <c r="AB20" s="3"/>
+        <v>25.25</v>
+      </c>
+      <c r="AB20" s="3">
+        <v>25.25</v>
+      </c>
       <c r="AC20" s="3">
-        <v>32.25</v>
+        <v>25.25</v>
       </c>
       <c r="AD20" s="13"/>
       <c r="AE20" s="13"/>
@@ -2662,7 +2691,9 @@
       <c r="U22" s="3">
         <v>0</v>
       </c>
-      <c r="V22" s="3"/>
+      <c r="V22" s="3">
+        <v>0</v>
+      </c>
       <c r="W22" s="3">
         <v>0</v>
       </c>
@@ -2986,17 +3017,19 @@
       <c r="Y26" s="13"/>
       <c r="Z26" s="13"/>
       <c r="AA26" s="5">
-        <v>100</v>
-      </c>
-      <c r="AB26" s="5"/>
+        <v>80</v>
+      </c>
+      <c r="AB26" s="5">
+        <v>80</v>
+      </c>
       <c r="AC26" s="5">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AD26" s="5">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AE26" s="5">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AF26" s="5">
         <v>76</v>
@@ -3137,17 +3170,19 @@
       <c r="Y28" s="13"/>
       <c r="Z28" s="13"/>
       <c r="AA28" s="5">
-        <v>100</v>
-      </c>
-      <c r="AB28" s="5"/>
+        <v>80</v>
+      </c>
+      <c r="AB28" s="5">
+        <v>80</v>
+      </c>
       <c r="AC28" s="5">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AD28" s="5">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AE28" s="5">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AF28" s="5">
         <v>76</v>
@@ -3253,7 +3288,7 @@
         <v>2</v>
       </c>
       <c r="C30" s="24">
-        <f>SUM(AA30:AF30,AH30:AK30)</f>
+        <f>SUM(AB30:AF30,AH30:AM30)</f>
         <v>285.60000000000002</v>
       </c>
       <c r="D30" s="21">
@@ -3287,39 +3322,43 @@
       <c r="X30" s="13"/>
       <c r="Y30" s="13"/>
       <c r="Z30" s="13"/>
-      <c r="AA30" s="5">
-        <v>32</v>
-      </c>
-      <c r="AB30" s="5"/>
+      <c r="AA30" s="13"/>
+      <c r="AB30" s="5">
+        <v>26</v>
+      </c>
       <c r="AC30" s="5">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="AD30" s="5">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="AE30" s="5">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="AF30" s="5">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="AG30" s="6" t="s">
         <v>21</v>
       </c>
       <c r="AH30" s="5">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="AI30" s="5">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="AJ30" s="5">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="AK30" s="5">
-        <v>29.6</v>
-      </c>
-      <c r="AL30" s="13"/>
-      <c r="AM30" s="13"/>
+        <v>26</v>
+      </c>
+      <c r="AL30" s="5">
+        <v>26</v>
+      </c>
+      <c r="AM30" s="5">
+        <v>25.6</v>
+      </c>
       <c r="AN30" s="13"/>
       <c r="AO30" s="13"/>
       <c r="AP30" s="13"/>
@@ -3412,7 +3451,7 @@
         <v>2</v>
       </c>
       <c r="C32" s="24">
-        <f>SUM(AC32:AF32,AH32:AL32)</f>
+        <f>SUM(AC32:AF32,AH32:AN32)</f>
         <v>43.3</v>
       </c>
       <c r="D32" s="21">
@@ -3449,37 +3488,41 @@
       <c r="AA32" s="6"/>
       <c r="AB32" s="6"/>
       <c r="AC32" s="8">
-        <v>4.8099999999999996</v>
+        <v>3.94</v>
       </c>
       <c r="AD32" s="8">
-        <v>4.8099999999999996</v>
+        <v>3.94</v>
       </c>
       <c r="AE32" s="8">
-        <v>4.8099999999999996</v>
+        <v>3.94</v>
       </c>
       <c r="AF32" s="8">
-        <v>4.8099999999999996</v>
+        <v>3.94</v>
       </c>
       <c r="AG32" s="6" t="s">
         <v>21</v>
       </c>
       <c r="AH32" s="8">
-        <v>4.8099999999999996</v>
+        <v>3.94</v>
       </c>
       <c r="AI32" s="8">
-        <v>4.8099999999999996</v>
+        <v>3.94</v>
       </c>
       <c r="AJ32" s="8">
-        <v>4.8099999999999996</v>
+        <v>3.94</v>
       </c>
       <c r="AK32" s="8">
-        <v>4.8099999999999996</v>
+        <v>3.94</v>
       </c>
       <c r="AL32" s="8">
-        <v>4.82</v>
-      </c>
-      <c r="AM32" s="8"/>
-      <c r="AN32" s="13"/>
+        <v>3.94</v>
+      </c>
+      <c r="AM32" s="8">
+        <v>3.94</v>
+      </c>
+      <c r="AN32" s="8">
+        <v>3.9</v>
+      </c>
       <c r="AO32" s="13"/>
       <c r="AP32" s="13"/>
       <c r="AQ32" s="13"/>
@@ -3571,7 +3614,7 @@
         <v>2</v>
       </c>
       <c r="C34" s="24">
-        <f>SUM(AD34:AF34,AH34:AN34)</f>
+        <f>SUM(AD34:AF34,AH34:AO34)</f>
         <v>43.3</v>
       </c>
       <c r="D34" s="21">
@@ -3609,37 +3652,41 @@
       <c r="AB34" s="6"/>
       <c r="AC34" s="6"/>
       <c r="AD34" s="8">
-        <v>4.8099999999999996</v>
+        <v>3.94</v>
       </c>
       <c r="AE34" s="8">
-        <v>4.8099999999999996</v>
+        <v>3.94</v>
       </c>
       <c r="AF34" s="8">
-        <v>4.8099999999999996</v>
+        <v>3.94</v>
       </c>
       <c r="AG34" s="6" t="s">
         <v>21</v>
       </c>
       <c r="AH34" s="8">
-        <v>4.8099999999999996</v>
+        <v>3.94</v>
       </c>
       <c r="AI34" s="8">
-        <v>4.8099999999999996</v>
+        <v>3.94</v>
       </c>
       <c r="AJ34" s="8">
-        <v>4.8099999999999996</v>
+        <v>3.94</v>
       </c>
       <c r="AK34" s="8">
-        <v>4.8099999999999996</v>
+        <v>3.94</v>
       </c>
       <c r="AL34" s="8">
-        <v>4.8099999999999996</v>
-      </c>
-      <c r="AM34" s="8"/>
+        <v>3.94</v>
+      </c>
+      <c r="AM34" s="8">
+        <v>3.94</v>
+      </c>
       <c r="AN34" s="8">
-        <v>4.82</v>
-      </c>
-      <c r="AO34" s="13"/>
+        <v>3.94</v>
+      </c>
+      <c r="AO34" s="8">
+        <v>3.9</v>
+      </c>
       <c r="AP34" s="13"/>
       <c r="AQ34" s="13"/>
       <c r="AR34" s="13"/>
@@ -3730,8 +3777,8 @@
         <v>2</v>
       </c>
       <c r="C36" s="24">
-        <f>SUM(AD36:AF36,AH36:AN36)</f>
-        <v>238.00000000000003</v>
+        <f>SUM(AD36:AF36,AH36:AO36)</f>
+        <v>237.99999999999997</v>
       </c>
       <c r="D36" s="21">
         <v>46097</v>
@@ -3768,37 +3815,41 @@
       <c r="AB36" s="6"/>
       <c r="AC36" s="6"/>
       <c r="AD36" s="8">
-        <v>26.4</v>
+        <v>21.6</v>
       </c>
       <c r="AE36" s="8">
-        <v>26.4</v>
+        <v>21.6</v>
       </c>
       <c r="AF36" s="8">
-        <v>26.4</v>
+        <v>21.6</v>
       </c>
       <c r="AG36" s="6" t="s">
         <v>21</v>
       </c>
       <c r="AH36" s="8">
-        <v>26.4</v>
+        <v>21.6</v>
       </c>
       <c r="AI36" s="8">
-        <v>26.4</v>
+        <v>21.6</v>
       </c>
       <c r="AJ36" s="8">
-        <v>26.4</v>
+        <v>21.6</v>
       </c>
       <c r="AK36" s="8">
-        <v>26.4</v>
+        <v>21.6</v>
       </c>
       <c r="AL36" s="8">
-        <v>26.4</v>
-      </c>
-      <c r="AM36" s="8"/>
+        <v>21.6</v>
+      </c>
+      <c r="AM36" s="8">
+        <v>21.6</v>
+      </c>
       <c r="AN36" s="8">
-        <v>26.8</v>
-      </c>
-      <c r="AO36" s="13"/>
+        <v>21.6</v>
+      </c>
+      <c r="AO36" s="8">
+        <v>22</v>
+      </c>
       <c r="AP36" s="13"/>
       <c r="AQ36" s="13"/>
       <c r="AR36" s="13"/>
@@ -3889,8 +3940,8 @@
         <v>2</v>
       </c>
       <c r="C38" s="24">
-        <f>SUM(AD38:AF38,AH38:AN38)</f>
-        <v>238.00000000000003</v>
+        <f>SUM(AD38:AF38,AH38:AO38)</f>
+        <v>237.99999999999997</v>
       </c>
       <c r="D38" s="21">
         <v>46097</v>
@@ -3927,37 +3978,41 @@
       <c r="AB38" s="6"/>
       <c r="AC38" s="6"/>
       <c r="AD38" s="8">
-        <v>26.4</v>
+        <v>21.6</v>
       </c>
       <c r="AE38" s="8">
-        <v>26.4</v>
+        <v>21.6</v>
       </c>
       <c r="AF38" s="8">
-        <v>26.4</v>
+        <v>21.6</v>
       </c>
       <c r="AG38" s="6" t="s">
         <v>21</v>
       </c>
       <c r="AH38" s="8">
-        <v>26.4</v>
+        <v>21.6</v>
       </c>
       <c r="AI38" s="8">
-        <v>26.4</v>
+        <v>21.6</v>
       </c>
       <c r="AJ38" s="8">
-        <v>26.4</v>
+        <v>21.6</v>
       </c>
       <c r="AK38" s="8">
-        <v>26.4</v>
+        <v>21.6</v>
       </c>
       <c r="AL38" s="8">
-        <v>26.4</v>
-      </c>
-      <c r="AM38" s="8"/>
+        <v>21.6</v>
+      </c>
+      <c r="AM38" s="8">
+        <v>21.6</v>
+      </c>
       <c r="AN38" s="8">
-        <v>26.8</v>
-      </c>
-      <c r="AO38" s="13"/>
+        <v>21.6</v>
+      </c>
+      <c r="AO38" s="8">
+        <v>22</v>
+      </c>
       <c r="AP38" s="13"/>
       <c r="AQ38" s="13"/>
       <c r="AR38" s="13"/>
@@ -4048,7 +4103,7 @@
         <v>2</v>
       </c>
       <c r="C40" s="24">
-        <f>SUM(AF40,AH40:AN40)</f>
+        <f>SUM(AF40,AH40:AO40)</f>
         <v>3</v>
       </c>
       <c r="D40" s="21">
@@ -4094,17 +4149,17 @@
         <v>21</v>
       </c>
       <c r="AH40" s="8"/>
-      <c r="AI40" s="8">
+      <c r="AI40" s="8"/>
+      <c r="AJ40" s="8"/>
+      <c r="AK40" s="8">
         <v>1</v>
       </c>
-      <c r="AJ40" s="8"/>
-      <c r="AK40" s="8"/>
       <c r="AL40" s="8"/>
       <c r="AM40" s="8"/>
-      <c r="AN40" s="8">
+      <c r="AN40" s="8"/>
+      <c r="AO40" s="8">
         <v>1</v>
       </c>
-      <c r="AO40" s="13"/>
       <c r="AP40" s="13"/>
       <c r="AQ40" s="13"/>
       <c r="AR40" s="13"/>
@@ -4196,7 +4251,7 @@
       </c>
       <c r="C42" s="24">
         <f>SUM(AD42:AF42,AH42:AO42)</f>
-        <v>255.99999999999997</v>
+        <v>234.30000000000004</v>
       </c>
       <c r="D42" s="21">
         <v>46097</v>
@@ -4233,40 +4288,44 @@
       <c r="AB42" s="6"/>
       <c r="AC42" s="6"/>
       <c r="AD42" s="8">
-        <v>25.6</v>
+        <v>21.3</v>
       </c>
       <c r="AE42" s="8">
-        <v>25.6</v>
+        <v>21.3</v>
       </c>
       <c r="AF42" s="8">
-        <v>25.6</v>
+        <v>21.3</v>
       </c>
       <c r="AG42" s="6" t="s">
         <v>21</v>
       </c>
       <c r="AH42" s="8">
-        <v>25.6</v>
+        <v>21.3</v>
       </c>
       <c r="AI42" s="8">
-        <v>25.6</v>
+        <v>21.3</v>
       </c>
       <c r="AJ42" s="8">
-        <v>25.6</v>
+        <v>21.3</v>
       </c>
       <c r="AK42" s="8">
-        <v>25.6</v>
+        <v>21.3</v>
       </c>
       <c r="AL42" s="8">
-        <v>25.6</v>
-      </c>
-      <c r="AM42" s="8"/>
+        <v>21.3</v>
+      </c>
+      <c r="AM42" s="8">
+        <v>21.3</v>
+      </c>
       <c r="AN42" s="8">
-        <v>25.6</v>
+        <v>21.3</v>
       </c>
       <c r="AO42" s="8">
-        <v>25.6</v>
-      </c>
-      <c r="AP42" s="13"/>
+        <v>21.3</v>
+      </c>
+      <c r="AP42" s="8">
+        <v>21.7</v>
+      </c>
       <c r="AQ42" s="13"/>
       <c r="AR42" s="13"/>
       <c r="AS42" s="13"/>
@@ -4418,7 +4477,9 @@
       <c r="AL44" s="8">
         <v>0</v>
       </c>
-      <c r="AM44" s="8"/>
+      <c r="AM44" s="8">
+        <v>0</v>
+      </c>
       <c r="AN44" s="8">
         <v>0</v>
       </c>
@@ -4513,7 +4574,7 @@
         <v>2</v>
       </c>
       <c r="C46" s="24">
-        <f>SUM(AO46)</f>
+        <f>SUM(AQ46)</f>
         <v>476</v>
       </c>
       <c r="D46" s="21">
@@ -4563,11 +4624,10 @@
       <c r="AL46" s="6"/>
       <c r="AM46" s="6"/>
       <c r="AN46" s="6"/>
-      <c r="AO46" s="8">
+      <c r="AP46" s="6"/>
+      <c r="AQ46" s="8">
         <v>476</v>
       </c>
-      <c r="AP46" s="6"/>
-      <c r="AQ46" s="6"/>
       <c r="AR46" s="6"/>
       <c r="AS46" s="6"/>
       <c r="AT46" s="6" t="s">
@@ -4656,7 +4716,7 @@
         <v>3</v>
       </c>
       <c r="C48" s="19">
-        <f>SUM(AP48:AQ48)</f>
+        <f>SUM(AQ48:AR48)</f>
         <v>126</v>
       </c>
       <c r="D48" s="21">
@@ -4707,13 +4767,13 @@
       <c r="AM48" s="13"/>
       <c r="AN48" s="13"/>
       <c r="AO48" s="13"/>
-      <c r="AP48" s="7">
-        <v>100</v>
-      </c>
+      <c r="AP48" s="13"/>
       <c r="AQ48" s="7">
-        <v>26</v>
-      </c>
-      <c r="AR48" s="4"/>
+        <v>63</v>
+      </c>
+      <c r="AR48" s="7">
+        <v>63</v>
+      </c>
       <c r="AS48" s="4"/>
       <c r="AT48" s="6" t="s">
         <v>21</v>
@@ -4777,7 +4837,7 @@
       <c r="AM49" s="13"/>
       <c r="AN49" s="13"/>
       <c r="AO49" s="13"/>
-      <c r="AP49" s="4"/>
+      <c r="AP49" s="13"/>
       <c r="AQ49" s="4"/>
       <c r="AR49" s="4"/>
       <c r="AS49" s="4"/>
@@ -4801,7 +4861,7 @@
         <v>3</v>
       </c>
       <c r="C50" s="19">
-        <f>SUM(AP50:AQ50)</f>
+        <f>SUM(AQ50:AR50)</f>
         <v>126</v>
       </c>
       <c r="D50" s="21">
@@ -4852,13 +4912,13 @@
       <c r="AM50" s="13"/>
       <c r="AN50" s="13"/>
       <c r="AO50" s="13"/>
-      <c r="AP50" s="7">
-        <v>100</v>
-      </c>
+      <c r="AP50" s="13"/>
       <c r="AQ50" s="7">
-        <v>26</v>
-      </c>
-      <c r="AR50" s="4"/>
+        <v>63</v>
+      </c>
+      <c r="AR50" s="7">
+        <v>63</v>
+      </c>
       <c r="AS50" s="4"/>
       <c r="AT50" s="6" t="s">
         <v>21</v>
@@ -4922,7 +4982,7 @@
       <c r="AM51" s="13"/>
       <c r="AN51" s="13"/>
       <c r="AO51" s="13"/>
-      <c r="AP51" s="4"/>
+      <c r="AP51" s="13"/>
       <c r="AQ51" s="4"/>
       <c r="AR51" s="4"/>
       <c r="AS51" s="4"/>
@@ -4946,7 +5006,7 @@
         <v>3</v>
       </c>
       <c r="C52" s="19">
-        <f>SUM(AP52:AQ52)</f>
+        <f>SUM(AQ52:AS52)</f>
         <v>75.599999999999994</v>
       </c>
       <c r="D52" s="21">
@@ -4997,14 +5057,16 @@
       <c r="AM52" s="13"/>
       <c r="AN52" s="13"/>
       <c r="AO52" s="13"/>
-      <c r="AP52" s="7">
-        <v>50</v>
-      </c>
+      <c r="AP52" s="13"/>
       <c r="AQ52" s="7">
-        <v>25.6</v>
-      </c>
-      <c r="AR52" s="6"/>
-      <c r="AS52" s="6"/>
+        <v>25.2</v>
+      </c>
+      <c r="AR52" s="7">
+        <v>25.2</v>
+      </c>
+      <c r="AS52" s="7">
+        <v>25.2</v>
+      </c>
       <c r="AT52" s="6" t="s">
         <v>21</v>
       </c>
@@ -5067,7 +5129,7 @@
       <c r="AM53" s="13"/>
       <c r="AN53" s="13"/>
       <c r="AO53" s="13"/>
-      <c r="AP53" s="6"/>
+      <c r="AP53" s="13"/>
       <c r="AQ53" s="6"/>
       <c r="AR53" s="6"/>
       <c r="AS53" s="6"/>
@@ -5091,8 +5153,8 @@
         <v>3</v>
       </c>
       <c r="C54" s="19">
-        <f>SUM(AQ54:AR54)</f>
-        <v>11.4</v>
+        <f>SUM(AR54:AS54,AV54)</f>
+        <v>11.399999999999999</v>
       </c>
       <c r="D54" s="21">
         <v>46097</v>
@@ -5142,21 +5204,23 @@
       <c r="AM54" s="13"/>
       <c r="AN54" s="13"/>
       <c r="AO54" s="13"/>
-      <c r="AP54" s="9"/>
-      <c r="AQ54" s="7">
-        <v>5.7</v>
-      </c>
+      <c r="AP54" s="13"/>
+      <c r="AQ54" s="9"/>
       <c r="AR54" s="7">
-        <v>5.7</v>
-      </c>
-      <c r="AS54" s="7"/>
+        <v>3.8</v>
+      </c>
+      <c r="AS54" s="7">
+        <v>3.8</v>
+      </c>
       <c r="AT54" s="6" t="s">
         <v>21</v>
       </c>
       <c r="AU54" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="AV54" s="6"/>
+      <c r="AV54" s="7">
+        <v>3.8</v>
+      </c>
       <c r="AW54" s="6"/>
       <c r="AX54" s="13"/>
       <c r="AY54" s="13"/>
@@ -5212,7 +5276,7 @@
       <c r="AM55" s="13"/>
       <c r="AN55" s="13"/>
       <c r="AO55" s="13"/>
-      <c r="AP55" s="6"/>
+      <c r="AP55" s="13"/>
       <c r="AQ55" s="6"/>
       <c r="AR55" s="6"/>
       <c r="AS55" s="6"/>
@@ -5236,8 +5300,8 @@
         <v>3</v>
       </c>
       <c r="C56" s="19">
-        <f>SUM(AV56,AR56)</f>
-        <v>11.4</v>
+        <f>SUM(AV56:AW56,AS56)</f>
+        <v>11.399999999999999</v>
       </c>
       <c r="D56" s="21">
         <v>46097</v>
@@ -5287,12 +5351,12 @@
       <c r="AM56" s="13"/>
       <c r="AN56" s="13"/>
       <c r="AO56" s="13"/>
-      <c r="AP56" s="9"/>
+      <c r="AP56" s="13"/>
       <c r="AQ56" s="9"/>
-      <c r="AR56" s="7">
-        <v>5.7</v>
-      </c>
-      <c r="AS56" s="7"/>
+      <c r="AR56" s="9"/>
+      <c r="AS56" s="7">
+        <v>3.8</v>
+      </c>
       <c r="AT56" s="6" t="s">
         <v>21</v>
       </c>
@@ -5300,9 +5364,11 @@
         <v>21</v>
       </c>
       <c r="AV56" s="7">
-        <v>5.7</v>
-      </c>
-      <c r="AW56" s="6"/>
+        <v>3.8</v>
+      </c>
+      <c r="AW56" s="7">
+        <v>3.8</v>
+      </c>
       <c r="AX56" s="13"/>
       <c r="AY56" s="13"/>
       <c r="AZ56" s="13"/>
@@ -5357,7 +5423,7 @@
       <c r="AM57" s="13"/>
       <c r="AN57" s="13"/>
       <c r="AO57" s="13"/>
-      <c r="AP57" s="6"/>
+      <c r="AP57" s="13"/>
       <c r="AQ57" s="6"/>
       <c r="AR57" s="6"/>
       <c r="AS57" s="6"/>
@@ -5381,7 +5447,7 @@
         <v>3</v>
       </c>
       <c r="C58" s="19">
-        <f>SUM(AV58,AR58)</f>
+        <f>SUM(AV58:AW58,AS58)</f>
         <v>63</v>
       </c>
       <c r="D58" s="21">
@@ -5432,12 +5498,12 @@
       <c r="AM58" s="13"/>
       <c r="AN58" s="13"/>
       <c r="AO58" s="13"/>
-      <c r="AP58" s="6"/>
+      <c r="AP58" s="13"/>
       <c r="AQ58" s="6"/>
-      <c r="AR58" s="10">
-        <v>40</v>
-      </c>
-      <c r="AS58" s="10"/>
+      <c r="AR58" s="6"/>
+      <c r="AS58" s="10">
+        <v>21</v>
+      </c>
       <c r="AT58" s="6" t="s">
         <v>21</v>
       </c>
@@ -5445,9 +5511,11 @@
         <v>21</v>
       </c>
       <c r="AV58" s="10">
-        <v>23</v>
-      </c>
-      <c r="AW58" s="6"/>
+        <v>21</v>
+      </c>
+      <c r="AW58" s="10">
+        <v>21</v>
+      </c>
       <c r="AX58" s="13"/>
       <c r="AY58" s="13"/>
       <c r="AZ58" s="13"/>
@@ -5502,7 +5570,7 @@
       <c r="AM59" s="13"/>
       <c r="AN59" s="13"/>
       <c r="AO59" s="13"/>
-      <c r="AP59" s="6"/>
+      <c r="AP59" s="13"/>
       <c r="AQ59" s="6"/>
       <c r="AR59" s="6"/>
       <c r="AS59" s="6"/>
@@ -5526,7 +5594,7 @@
         <v>3</v>
       </c>
       <c r="C60" s="19">
-        <f>SUM(AV60,AR60)</f>
+        <f>SUM(AV60:AW60,AS60)</f>
         <v>63</v>
       </c>
       <c r="D60" s="21">
@@ -5577,12 +5645,12 @@
       <c r="AM60" s="13"/>
       <c r="AN60" s="13"/>
       <c r="AO60" s="13"/>
-      <c r="AP60" s="6"/>
+      <c r="AP60" s="13"/>
       <c r="AQ60" s="6"/>
-      <c r="AR60" s="10">
-        <v>40</v>
-      </c>
-      <c r="AS60" s="10"/>
+      <c r="AR60" s="6"/>
+      <c r="AS60" s="10">
+        <v>21</v>
+      </c>
       <c r="AT60" s="6" t="s">
         <v>21</v>
       </c>
@@ -5590,9 +5658,11 @@
         <v>21</v>
       </c>
       <c r="AV60" s="10">
-        <v>23</v>
-      </c>
-      <c r="AW60" s="6"/>
+        <v>21</v>
+      </c>
+      <c r="AW60" s="10">
+        <v>21</v>
+      </c>
       <c r="AX60" s="13"/>
       <c r="AY60" s="13"/>
       <c r="AZ60" s="13"/>
@@ -5671,7 +5741,7 @@
         <v>3</v>
       </c>
       <c r="C62" s="19">
-        <f>SUM(AV62)</f>
+        <f>SUM(AW62)</f>
         <v>1</v>
       </c>
       <c r="D62" s="21">
@@ -5732,10 +5802,9 @@
       <c r="AU62" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="AV62" s="10">
+      <c r="AW62" s="10">
         <v>1</v>
       </c>
-      <c r="AW62" s="6"/>
       <c r="AX62" s="13"/>
       <c r="AY62" s="13"/>
       <c r="AZ62" s="13"/>
@@ -5814,7 +5883,7 @@
         <v>3</v>
       </c>
       <c r="C64" s="19">
-        <f>SUM(AV64:AW64)</f>
+        <f>SUM(AV64:AX64)</f>
         <v>55</v>
       </c>
       <c r="D64" s="21">
@@ -5876,12 +5945,14 @@
         <v>21</v>
       </c>
       <c r="AV64" s="10">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="AW64" s="10">
-        <v>25</v>
-      </c>
-      <c r="AX64" s="13"/>
+        <v>18</v>
+      </c>
+      <c r="AX64" s="10">
+        <v>18</v>
+      </c>
       <c r="AY64" s="13"/>
       <c r="AZ64" s="13"/>
       <c r="BA64" s="13"/>

</xml_diff>